<commit_message>
Google Ads: vrijgezellenfeest- en teamuitjecampagne erbij, alle vier in één importbestand, geen brede zoekwoorden
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/seo/ads/merkcampagne/merkcampagne-overzicht.xlsx
+++ b/tools/seo/ads/merkcampagne/merkcampagne-overzicht.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X69"/>
+  <dimension ref="A1:X82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8836,6 +8836,1592 @@
       <c r="X69" t="inlineStr">
         <is>
           <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie groep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Utrecht</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/vrijgezellenfeest-utrecht/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>vrijgezellenfeest utrecht, vrijgezellenuitje utrecht, vrijgezellendag utrecht</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Utrecht</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Actief Vrijgezellenuitje</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Utrecht</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Wie Ontsnapt aan de Hunters?</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Vanaf 8 Personen</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Ontsnappen</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Aanvragen</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Origineel Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Voor Bruid én Bruidegom</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest in Utrecht: ontsnap 90 minuten aan echte live Hunters in de stad.</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en samenwerken. Een actief uitje voor groepen vanaf 8 personen.</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie feest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Rotterdam</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/vrijgezellenfeest-rotterdam-perfect-groepen/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>vrijgezellenfeest rotterdam, vrijgezellenuitje rotterdam, vrijgezellendag rotterdam</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Rotterdam</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Actief Vrijgezellenuitje</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Rotterdam</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Wie Ontsnapt aan de Hunters?</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Vanaf 8 Personen</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Ontsnappen</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Aanvragen</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Origineel Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>Voor Bruid én Bruidegom</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest in Rotterdam: ontsnap 90 minuten aan echte live Hunters in de stad.</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en samenwerken. Een actief uitje voor groepen vanaf 8 personen.</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie feest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Amsterdam</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/vrijgezellenfeest-amsterdam/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>vrijgezellenfeest amsterdam, vrijgezellenuitje amsterdam, vrijgezellendag amsterdam</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Amsterdam</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Actief Vrijgezellenuitje</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Amsterdam</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Wie Ontsnapt aan de Hunters?</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Vanaf 8 Personen</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Ontsnappen</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Aanvragen</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Origineel Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>Voor Bruid én Bruidegom</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest in Amsterdam: ontsnap 90 minuten aan echte live Hunters in de stad.</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en samenwerken. Een actief uitje voor groepen vanaf 8 personen.</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie feest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Groningen</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/vrijgezellenfeest-groningen-het-meest-actieve-avontuur-voor-de-bruidegom/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>vrijgezellenfeest groningen, vrijgezellenuitje groningen, vrijgezellendag groningen</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Groningen</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Actief Vrijgezellenuitje</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Groningen</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>Wie Ontsnapt aan de Hunters?</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Vanaf 8 Personen</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Ontsnappen</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Aanvragen</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Origineel Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Voor Bruid én Bruidegom</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest in Groningen: ontsnap 90 minuten aan echte live Hunters in de stad.</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en samenwerken. Een actief uitje voor groepen vanaf 8 personen.</t>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie feest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Amersfoort</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/vrijgezellenfeest-amersfoort-wie-van-jullie-weet-te-ontsnappen-aan-de-hunters/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>vrijgezellenfeest amersfoort, vrijgezellenuitje amersfoort, vrijgezellendag amersfoort</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Amersfoort</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Actief Vrijgezellenuitje</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Amersfoort</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Wie Ontsnapt aan de Hunters?</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>Vanaf 8 Personen</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Ontsnappen</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Aanvragen</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Origineel Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>Voor Bruid én Bruidegom</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest in Amersfoort: ontsnap 90 minuten aan echte live Hunters in de stad.</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en samenwerken. Een actief uitje voor groepen vanaf 8 personen.</t>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie feest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Zwolle</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/vrijgezellenfeest-zwolle/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>vrijgezellenfeest zwolle, vrijgezellenuitje zwolle, vrijgezellendag zwolle</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Zwolle</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Actief Vrijgezellenuitje</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Zwolle</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>Wie Ontsnapt aan de Hunters?</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>Vanaf 8 Personen</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Ontsnappen</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Aanvragen</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Origineel Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>Voor Bruid én Bruidegom</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest in Zwolle: ontsnap 90 minuten aan echte live Hunters in de stad.</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en samenwerken. Een actief uitje voor groepen vanaf 8 personen.</t>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie feest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Nijmegen</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/vrijgezellenfeest-nijmegen-beleef-een-onvergetelijk-avontuur-met-escape-game-the-hunt/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>vrijgezellenfeest nijmegen, vrijgezellenuitje nijmegen, vrijgezellendag nijmegen</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Nijmegen</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Actief Vrijgezellenuitje</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Nijmegen</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>Wie Ontsnapt aan de Hunters?</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Vanaf 8 Personen</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Ontsnappen</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Aanvragen</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Origineel Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>Voor Bruid én Bruidegom</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest in Nijmegen: ontsnap 90 minuten aan echte live Hunters in de stad.</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en samenwerken. Een actief uitje voor groepen vanaf 8 personen.</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie feest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Maastricht</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/vrijgezellenfeest-maastricht/</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>vrijgezellenfeest maastricht, vrijgezellenuitje maastricht, vrijgezellendag maastricht</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest Maastricht</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Actief Vrijgezellenuitje</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Maastricht</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Wie Ontsnapt aan de Hunters?</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Vanaf 8 Personen</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Ontsnappen</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Aanvragen</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Origineel Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>Voor Bruid én Bruidegom</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>Vrijgezellenfeest in Maastricht: ontsnap 90 minuten aan echte live Hunters in de stad.</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en samenwerken. Een actief uitje voor groepen vanaf 8 personen.</t>
+        </is>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum aan voor jullie feest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>The Hunt - Teamuitje</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje Groningen</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/bedrijfsuitje-groningen-combineer-stad/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>bedrijfsuitje groningen</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje Groningen</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Teamuitje met Live Hunters</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Teamuitje Groningen</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Teambuilding in de Buitenlucht</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Van 8 tot 200 Collega's</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Samenwerken</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Groningen</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Offerte Aanvragen</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Ook Op Maat Mogelijk</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje in Groningen: ontsnap 90 minuten met je collega's aan echte live Hunters.</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en strategie: teambuilding die energie geeft. Van 8 tot 200 personen.</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum en offerte aan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>The Hunt - Teamuitje</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Teamuitje Zwolle</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/teamuitje-bedrijfsuitje-zwolle/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>teamuitje zwolle</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Teamuitje Zwolle</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Teamuitje met Live Hunters</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje Zwolle</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Teambuilding in de Buitenlucht</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Van 8 tot 200 Collega's</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Samenwerken</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Zwolle</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Offerte Aanvragen</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Ook Op Maat Mogelijk</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>Teamuitje in Zwolle: ontsnap 90 minuten met je collega's aan echte live Hunters.</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en strategie: teambuilding die energie geeft. Van 8 tot 200 personen.</t>
+        </is>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum en offerte aan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>The Hunt - Teamuitje</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Teamuitje Tilburg</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/teamuitje-tilburg-organiseren-beleef-90-minuten-actie-met-the-hunt/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>teamuitje tilburg</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Teamuitje Tilburg</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Teamuitje met Live Hunters</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje Tilburg</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Teambuilding in de Buitenlucht</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>Van 8 tot 200 Collega's</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Samenwerken</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Tilburg</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Offerte Aanvragen</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Ook Op Maat Mogelijk</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>Teamuitje in Tilburg: ontsnap 90 minuten met je collega's aan echte live Hunters.</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en strategie: teambuilding die energie geeft. Van 8 tot 200 personen.</t>
+        </is>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum en offerte aan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>The Hunt - Teamuitje</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje Enschede</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/teamuitje-bedrijfsuitje-enschede/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>bedrijfsuitje enschede</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje Enschede</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Teamuitje met Live Hunters</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Teamuitje Enschede</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Teambuilding in de Buitenlucht</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Van 8 tot 200 Collega's</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Samenwerken</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Enschede</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Offerte Aanvragen</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Ook Op Maat Mogelijk</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje in Enschede: ontsnap 90 minuten met je collega's aan echte live Hunters.</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en strategie: teambuilding die energie geeft. Van 8 tot 200 personen.</t>
+        </is>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum en offerte aan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>The Hunt - Teamuitje</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Teamuitje + Bedrijfsuitje Leeuwarden</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://escapegamethehunt.nl/teamuitje-bedrijfsuitje-leeuwarden/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>teamuitje leeuwarden, bedrijfsuitje leeuwarden</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Teamuitje Leeuwarden</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Ontsnap aan Live Hunters</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Echte Hunters Jagen op Jullie</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Teamuitje met Live Hunters</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Bedrijfsuitje Leeuwarden</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Teambuilding in de Buitenlucht</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>90 Minuten Pure Spanning</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>Escape Game The Hunt</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Van 8 tot 200 Collega's</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Puzzelen, Rennen, Samenwerken</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Outdoor Escape in Leeuwarden</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Live Hunters op Jullie Hielen</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>Vrijblijvend Offerte Aanvragen</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>De Stad Is Jullie Speelveld</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Ook Op Maat Mogelijk</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>Teamuitje in Leeuwarden: ontsnap 90 minuten met je collega's aan echte live Hunters.</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>Geen kamer maar de hele stad als speelveld. Live Hunters zitten jullie op de hielen.</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>Puzzelen, rennen en strategie: teambuilding die energie geeft. Van 8 tot 200 personen.</t>
+        </is>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>Dé escape game met live Hunters. Vraag vrijblijvend een datum en offerte aan.</t>
         </is>
       </c>
     </row>
@@ -8850,7 +10436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8930,8 +10516,54 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>The Hunt - Vrijgezellenfeest</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>vacature, werken bij, escape hunt, gratis, kinderfeestje, kinderen</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
+        <is>
+          <t>The Hunt - Teamuitje</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>vacature, werken bij, escape hunt, gratis, kinderfeestje, kinderen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Alle campagnes: alleen Google Zoeken (geen partners/display), Nederlands, heel Nederland, handmatige CPC, status Gepauzeerd.</t>
         </is>

</xml_diff>